<commit_message>
Atualização automática: 2026-07-01 15:26
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -13332,7 +13332,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>31/07/2026</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -13364,8 +13364,8 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 30/06/2026 
-AINDA NÃO HOUVE A REUNIÃO DE IMPLANTAÇÃO - Data Comentário: 10/06/2026 16:18</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+ainda não foi realizado as implantações - Data Comentário: 01/07/2026 13:38</t>
         </is>
       </c>
       <c r="V129" t="inlineStr"/>
@@ -13439,7 +13439,11 @@
       <c r="L130" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="M130" t="inlineStr"/>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N130" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -13469,7 +13473,8 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6962; Tarefa Incluida: 11617; Vencimento: 17/06/2026 00:00:00; UsuarioResponsavel: pvolpe - Data Comentário: 17/06/2026 11:09</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+ainda não foi realizado as implantações - Data Comentário: 01/07/2026 13:38</t>
         </is>
       </c>
       <c r="V130" t="inlineStr"/>
@@ -13543,7 +13548,11 @@
       <c r="L131" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="M131" t="inlineStr"/>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="N131" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -13573,7 +13582,8 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6963; Tarefa Incluida: 11617; Vencimento: 17/06/2026 00:00:00; UsuarioResponsavel: pvolpe - Data Comentário: 17/06/2026 11:09</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 31/07/2026 
+ainda não foi realizado as implantações - Data Comentário: 01/07/2026 13:38</t>
         </is>
       </c>
       <c r="V131" t="inlineStr"/>
@@ -78659,11 +78669,11 @@
     </row>
     <row r="784">
       <c r="A784" t="n">
-        <v>6358</v>
+        <v>6548</v>
       </c>
       <c r="B784" t="inlineStr">
         <is>
-          <t>QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA</t>
+          <t>GOIAS SILAGEM LTDA</t>
         </is>
       </c>
       <c r="C784" t="inlineStr">
@@ -78708,7 +78718,7 @@
       </c>
       <c r="M784" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="N784" t="inlineStr">
@@ -78717,11 +78727,11 @@
         </is>
       </c>
       <c r="O784" t="n">
-        <v>18096517</v>
+        <v>18096231</v>
       </c>
       <c r="P784" t="inlineStr">
         <is>
-          <t>Emylle Souza</t>
+          <t>Thais Souza</t>
         </is>
       </c>
       <c r="Q784" t="inlineStr">
@@ -78735,12 +78745,12 @@
       </c>
       <c r="T784" t="inlineStr">
         <is>
-          <t>MACHADO</t>
+          <t>GOIAS SILAGEM</t>
         </is>
       </c>
       <c r="U784" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 14/07/2026 - Data Comentário: 01/07/2026 09:04</t>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista   Previsão para conclusão dia 02/07/2026 - Data Comentário: 01/07/2026 09:36</t>
         </is>
       </c>
       <c r="V784" t="inlineStr"/>
@@ -78759,17 +78769,17 @@
       </c>
       <c r="AF784" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Erika Santana</t>
         </is>
       </c>
     </row>
     <row r="785">
       <c r="A785" t="n">
-        <v>6548</v>
+        <v>6627</v>
       </c>
       <c r="B785" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM LTDA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C785" t="inlineStr">
@@ -78784,7 +78794,7 @@
       </c>
       <c r="E785" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F785" t="inlineStr">
@@ -78812,22 +78822,18 @@
       <c r="L785" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="M785" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
+      <c r="M785" t="inlineStr"/>
       <c r="N785" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O785" t="n">
-        <v>18096231</v>
+        <v>18096484</v>
       </c>
       <c r="P785" t="inlineStr">
         <is>
-          <t>Thais Souza</t>
+          <t>Nathalia Lourenco</t>
         </is>
       </c>
       <c r="Q785" t="inlineStr">
@@ -78841,12 +78847,12 @@
       </c>
       <c r="T785" t="inlineStr">
         <is>
-          <t>GOIAS SILAGEM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U785" t="inlineStr">
         <is>
-          <t>Atraso da Operação, processo em elaboração conforme data prevista   Previsão para conclusão dia 02/07/2026 - Data Comentário: 01/07/2026 09:36</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 24/06/2026 12:07:35. - Data Comentário: 24/06/2026 12:06</t>
         </is>
       </c>
       <c r="V785" t="inlineStr"/>
@@ -78856,8 +78862,16 @@
       <c r="Z785" t="inlineStr"/>
       <c r="AA785" t="inlineStr"/>
       <c r="AB785" t="inlineStr"/>
-      <c r="AC785" t="inlineStr"/>
-      <c r="AD785" t="inlineStr"/>
+      <c r="AC785" t="inlineStr">
+        <is>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 25/06/2026. - Data Comentário: 24/06/2026 12:06</t>
+        </is>
+      </c>
+      <c r="AD785" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
       <c r="AE785" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -78865,17 +78879,17 @@
       </c>
       <c r="AF785" t="inlineStr">
         <is>
-          <t>Erika Santana</t>
+          <t>Isabella Nascimento</t>
         </is>
       </c>
     </row>
     <row r="786">
       <c r="A786" t="n">
-        <v>6627</v>
+        <v>5617</v>
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
@@ -78890,7 +78904,7 @@
       </c>
       <c r="E786" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F786" t="inlineStr">
@@ -78899,14 +78913,14 @@
         </is>
       </c>
       <c r="G786" t="n">
-        <v>7875</v>
+        <v>7874</v>
       </c>
       <c r="H786" t="n">
         <v>0</v>
       </c>
       <c r="I786" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL INDUSTRIA</t>
+          <t>CTB - CONTÁBIL VAREJO</t>
         </is>
       </c>
       <c r="J786" t="inlineStr">
@@ -78918,18 +78932,22 @@
       <c r="L786" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="M786" t="inlineStr"/>
+      <c r="M786" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
       <c r="N786" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O786" t="n">
-        <v>18096484</v>
+        <v>17407858</v>
       </c>
       <c r="P786" t="inlineStr">
         <is>
-          <t>Nathalia Lourenco</t>
+          <t>Jackson Silva</t>
         </is>
       </c>
       <c r="Q786" t="inlineStr">
@@ -78943,12 +78961,12 @@
       </c>
       <c r="T786" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U786" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 24/06/2026 12:07:35. - Data Comentário: 24/06/2026 12:06</t>
+          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 30/06/2026 - Data Comentário: 26/06/2026 14:11</t>
         </is>
       </c>
       <c r="V786" t="inlineStr"/>
@@ -78958,16 +78976,8 @@
       <c r="Z786" t="inlineStr"/>
       <c r="AA786" t="inlineStr"/>
       <c r="AB786" t="inlineStr"/>
-      <c r="AC786" t="inlineStr">
-        <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 25/06/2026. - Data Comentário: 24/06/2026 12:06</t>
-        </is>
-      </c>
-      <c r="AD786" t="inlineStr">
-        <is>
-          <t>25/06/2026</t>
-        </is>
-      </c>
+      <c r="AC786" t="inlineStr"/>
+      <c r="AD786" t="inlineStr"/>
       <c r="AE786" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -78975,17 +78985,17 @@
       </c>
       <c r="AF786" t="inlineStr">
         <is>
-          <t>Isabella Nascimento</t>
+          <t>Edileide Dias</t>
         </is>
       </c>
     </row>
     <row r="787">
       <c r="A787" t="n">
-        <v>5617</v>
+        <v>6224</v>
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -79005,7 +79015,7 @@
       </c>
       <c r="F787" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G787" t="n">
@@ -79039,7 +79049,7 @@
         </is>
       </c>
       <c r="O787" t="n">
-        <v>17407858</v>
+        <v>17206041</v>
       </c>
       <c r="P787" t="inlineStr">
         <is>
@@ -79087,11 +79097,11 @@
     </row>
     <row r="788">
       <c r="A788" t="n">
-        <v>6224</v>
+        <v>6704</v>
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
@@ -79111,7 +79121,7 @@
       </c>
       <c r="F788" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G788" t="n">
@@ -79134,22 +79144,18 @@
       <c r="L788" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="M788" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
-        </is>
-      </c>
+      <c r="M788" t="inlineStr"/>
       <c r="N788" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O788" t="n">
-        <v>17206041</v>
+        <v>18096764</v>
       </c>
       <c r="P788" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q788" t="inlineStr">
@@ -79163,12 +79169,12 @@
       </c>
       <c r="T788" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U788" t="inlineStr">
         <is>
-          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 30/06/2026 - Data Comentário: 26/06/2026 14:11</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:27:33. - Data Comentário: 29/06/2026 09:26</t>
         </is>
       </c>
       <c r="V788" t="inlineStr"/>
@@ -79178,8 +79184,16 @@
       <c r="Z788" t="inlineStr"/>
       <c r="AA788" t="inlineStr"/>
       <c r="AB788" t="inlineStr"/>
-      <c r="AC788" t="inlineStr"/>
-      <c r="AD788" t="inlineStr"/>
+      <c r="AC788" t="inlineStr">
+        <is>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:26</t>
+        </is>
+      </c>
+      <c r="AD788" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
       <c r="AE788" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -79187,17 +79201,17 @@
       </c>
       <c r="AF788" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" t="n">
-        <v>6704</v>
+        <v>6705</v>
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
@@ -79207,7 +79221,7 @@
       </c>
       <c r="D789" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E789" t="inlineStr">
@@ -79221,7 +79235,7 @@
         </is>
       </c>
       <c r="G789" t="n">
-        <v>7874</v>
+        <v>9762</v>
       </c>
       <c r="H789" t="n">
         <v>0</v>
@@ -79233,7 +79247,7 @@
       </c>
       <c r="J789" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>Movimento - Analise de Balanço Simples Nacional</t>
         </is>
       </c>
       <c r="K789" t="inlineStr"/>
@@ -79247,7 +79261,7 @@
         </is>
       </c>
       <c r="O789" t="n">
-        <v>18096764</v>
+        <v>18096936</v>
       </c>
       <c r="P789" t="inlineStr">
         <is>
@@ -79270,7 +79284,7 @@
       </c>
       <c r="U789" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:27:33. - Data Comentário: 29/06/2026 09:26</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:24:47. - Data Comentário: 29/06/2026 09:23</t>
         </is>
       </c>
       <c r="V789" t="inlineStr"/>
@@ -79282,7 +79296,7 @@
       <c r="AB789" t="inlineStr"/>
       <c r="AC789" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:26</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:23</t>
         </is>
       </c>
       <c r="AD789" t="inlineStr">
@@ -79303,11 +79317,11 @@
     </row>
     <row r="790">
       <c r="A790" t="n">
-        <v>6705</v>
+        <v>6279</v>
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -79317,7 +79331,7 @@
       </c>
       <c r="D790" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E790" t="inlineStr">
@@ -79327,41 +79341,41 @@
       </c>
       <c r="F790" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G790" t="n">
-        <v>9762</v>
+        <v>5800</v>
       </c>
       <c r="H790" t="n">
-        <v>0</v>
+        <v>5776</v>
       </c>
       <c r="I790" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J790" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Simples Nacional</t>
+          <t>CCT Lançamento Sd.508</t>
         </is>
       </c>
       <c r="K790" t="inlineStr"/>
       <c r="L790" s="1" t="n">
-        <v>46198</v>
+        <v>46203</v>
       </c>
       <c r="M790" t="inlineStr"/>
       <c r="N790" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>00/2026</t>
         </is>
       </c>
       <c r="O790" t="n">
-        <v>18096936</v>
+        <v>18087241</v>
       </c>
       <c r="P790" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Vitor Guedes</t>
         </is>
       </c>
       <c r="Q790" t="inlineStr">
@@ -79371,16 +79385,16 @@
       </c>
       <c r="R790" t="inlineStr"/>
       <c r="S790" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T790" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U790" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:24:47. - Data Comentário: 29/06/2026 09:23</t>
+          <t>8. Serviços Suspensos. - Data Comentário: 30/06/2026 17:29</t>
         </is>
       </c>
       <c r="V790" t="inlineStr"/>
@@ -79392,12 +79406,12 @@
       <c r="AB790" t="inlineStr"/>
       <c r="AC790" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:23</t>
+          <t>Aguardando liberação do sindicato - Data Comentário: 18/05/2026 17:19</t>
         </is>
       </c>
       <c r="AD790" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="AE790" t="inlineStr">
@@ -79407,17 +79421,17 @@
       </c>
       <c r="AF790" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" t="n">
-        <v>6279</v>
+        <v>6627</v>
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -79427,51 +79441,55 @@
       </c>
       <c r="D791" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G791" t="n">
-        <v>5800</v>
+        <v>7026</v>
       </c>
       <c r="H791" t="n">
-        <v>5776</v>
+        <v>0</v>
       </c>
       <c r="I791" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J791" t="inlineStr">
         <is>
-          <t>CCT Lançamento Sd.508</t>
+          <t>Movimento - Sistema de Análise</t>
         </is>
       </c>
       <c r="K791" t="inlineStr"/>
       <c r="L791" s="1" t="n">
-        <v>46203</v>
-      </c>
-      <c r="M791" t="inlineStr"/>
+        <v>46167</v>
+      </c>
+      <c r="M791" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
       <c r="N791" t="inlineStr">
         <is>
-          <t>00/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O791" t="n">
-        <v>18087241</v>
+        <v>18048469</v>
       </c>
       <c r="P791" t="inlineStr">
         <is>
-          <t>Vitor Guedes</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="Q791" t="inlineStr">
@@ -79481,16 +79499,17 @@
       </c>
       <c r="R791" t="inlineStr"/>
       <c r="S791" t="n">
-        <v>1</v>
+        <v>37</v>
       </c>
       <c r="T791" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U791" t="inlineStr">
         <is>
-          <t>8. Serviços Suspensos. - Data Comentário: 30/06/2026 17:29</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 26/06/2026 
+OPERAÇÃO X GC VALIDANDO COM SYS ANALISE - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V791" t="inlineStr"/>
@@ -79502,12 +79521,12 @@
       <c r="AB791" t="inlineStr"/>
       <c r="AC791" t="inlineStr">
         <is>
-          <t>Aguardando liberação do sindicato - Data Comentário: 18/05/2026 17:19</t>
+          <t>Operação e GC validando as informações errôneas no sistema de análise - Data Comentário: 24/06/2026 14:39</t>
         </is>
       </c>
       <c r="AD791" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="AE791" t="inlineStr">
@@ -79515,19 +79534,15 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AF791" t="inlineStr">
-        <is>
-          <t>David Bragança</t>
-        </is>
-      </c>
+      <c r="AF791" t="inlineStr"/>
     </row>
     <row r="792">
       <c r="A792" t="n">
-        <v>6627</v>
+        <v>6224</v>
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -79542,50 +79557,46 @@
       </c>
       <c r="E792" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G792" t="n">
-        <v>7026</v>
+        <v>1802</v>
       </c>
       <c r="H792" t="n">
         <v>0</v>
       </c>
       <c r="I792" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J792" t="inlineStr">
         <is>
-          <t>Movimento - Sistema de Análise</t>
+          <t>Est - ICMS RPA - CÓD. 046-2</t>
         </is>
       </c>
       <c r="K792" t="inlineStr"/>
       <c r="L792" s="1" t="n">
-        <v>46167</v>
-      </c>
-      <c r="M792" t="inlineStr">
-        <is>
-          <t>26/06/2026</t>
-        </is>
-      </c>
+        <v>46182</v>
+      </c>
+      <c r="M792" t="inlineStr"/>
       <c r="N792" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O792" t="n">
-        <v>18048469</v>
+        <v>17688680</v>
       </c>
       <c r="P792" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q792" t="inlineStr">
@@ -79595,17 +79606,16 @@
       </c>
       <c r="R792" t="inlineStr"/>
       <c r="S792" t="n">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="T792" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U792" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 26/06/2026 
-OPERAÇÃO X GC VALIDANDO COM SYS ANALISE - Data Comentário: 25/06/2026 16:00</t>
+          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V792" t="inlineStr"/>
@@ -79617,7 +79627,7 @@
       <c r="AB792" t="inlineStr"/>
       <c r="AC792" t="inlineStr">
         <is>
-          <t>Operação e GC validando as informações errôneas no sistema de análise - Data Comentário: 24/06/2026 14:39</t>
+          <t>Atraso por parte do cliente, GC e GM acionado - CA03 - Data Comentário: 25/06/2026 18:14</t>
         </is>
       </c>
       <c r="AD792" t="inlineStr">
@@ -79627,10 +79637,14 @@
       </c>
       <c r="AE792" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AF792" t="inlineStr"/>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AF792" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="n">
@@ -79662,7 +79676,7 @@
         </is>
       </c>
       <c r="G793" t="n">
-        <v>1802</v>
+        <v>1808</v>
       </c>
       <c r="H793" t="n">
         <v>0</v>
@@ -79674,12 +79688,12 @@
       </c>
       <c r="J793" t="inlineStr">
         <is>
-          <t>Est - ICMS RPA - CÓD. 046-2</t>
+          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
         </is>
       </c>
       <c r="K793" t="inlineStr"/>
       <c r="L793" s="1" t="n">
-        <v>46182</v>
+        <v>46195</v>
       </c>
       <c r="M793" t="inlineStr"/>
       <c r="N793" t="inlineStr">
@@ -79688,7 +79702,7 @@
         </is>
       </c>
       <c r="O793" t="n">
-        <v>17688680</v>
+        <v>17688690</v>
       </c>
       <c r="P793" t="inlineStr">
         <is>
@@ -79702,7 +79716,7 @@
       </c>
       <c r="R793" t="inlineStr"/>
       <c r="S793" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="T793" t="inlineStr">
         <is>
@@ -79711,7 +79725,7 @@
       </c>
       <c r="U793" t="inlineStr">
         <is>
-          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
+          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
         </is>
       </c>
       <c r="V793" t="inlineStr"/>
@@ -79723,7 +79737,7 @@
       <c r="AB793" t="inlineStr"/>
       <c r="AC793" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionado - CA03 - Data Comentário: 25/06/2026 18:14</t>
+          <t>Atraso por parte do cliente, GC e GM acionados - Data Comentário: 25/06/2026 18:14</t>
         </is>
       </c>
       <c r="AD793" t="inlineStr">
@@ -79744,11 +79758,11 @@
     </row>
     <row r="794">
       <c r="A794" t="n">
-        <v>6224</v>
+        <v>6404</v>
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
@@ -79758,7 +79772,7 @@
       </c>
       <c r="D794" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E794" t="inlineStr">
@@ -79768,41 +79782,45 @@
       </c>
       <c r="F794" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G794" t="n">
-        <v>1808</v>
+        <v>11001</v>
       </c>
       <c r="H794" t="n">
         <v>0</v>
       </c>
       <c r="I794" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J794" t="inlineStr">
         <is>
-          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
+          <t>Movimento - Analise de Balanço Lucro Presumido</t>
         </is>
       </c>
       <c r="K794" t="inlineStr"/>
       <c r="L794" s="1" t="n">
-        <v>46195</v>
-      </c>
-      <c r="M794" t="inlineStr"/>
+        <v>46202</v>
+      </c>
+      <c r="M794" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
       <c r="N794" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O794" t="n">
-        <v>17688690</v>
+        <v>16962451</v>
       </c>
       <c r="P794" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="Q794" t="inlineStr">
@@ -79812,16 +79830,17 @@
       </c>
       <c r="R794" t="inlineStr"/>
       <c r="S794" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="T794" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U794" t="inlineStr">
         <is>
-          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
+Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
         </is>
       </c>
       <c r="V794" t="inlineStr"/>
@@ -79833,32 +79852,28 @@
       <c r="AB794" t="inlineStr"/>
       <c r="AC794" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionados - Data Comentário: 25/06/2026 18:14</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:45</t>
         </is>
       </c>
       <c r="AD794" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="AE794" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AF794" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AF794" t="inlineStr"/>
     </row>
     <row r="795">
       <c r="A795" t="n">
-        <v>6404</v>
+        <v>5417</v>
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
@@ -79868,7 +79883,7 @@
       </c>
       <c r="D795" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E795" t="inlineStr">
@@ -79878,11 +79893,11 @@
       </c>
       <c r="F795" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G795" t="n">
-        <v>11001</v>
+        <v>7877</v>
       </c>
       <c r="H795" t="n">
         <v>0</v>
@@ -79894,29 +79909,25 @@
       </c>
       <c r="J795" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Presumido</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K795" t="inlineStr"/>
       <c r="L795" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="M795" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
+      <c r="M795" t="inlineStr"/>
       <c r="N795" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O795" t="n">
-        <v>16962451</v>
+        <v>17399327</v>
       </c>
       <c r="P795" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Sergio Fernandes</t>
         </is>
       </c>
       <c r="Q795" t="inlineStr">
@@ -79930,13 +79941,12 @@
       </c>
       <c r="T795" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U795" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
-Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 30/06/2026 18:03:37. - Data Comentário: 30/06/2026 18:02</t>
         </is>
       </c>
       <c r="V795" t="inlineStr"/>
@@ -79948,7 +79958,7 @@
       <c r="AB795" t="inlineStr"/>
       <c r="AC795" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:45</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 18:02</t>
         </is>
       </c>
       <c r="AD795" t="inlineStr">
@@ -79965,11 +79975,11 @@
     </row>
     <row r="796">
       <c r="A796" t="n">
-        <v>5417</v>
+        <v>6224</v>
       </c>
       <c r="B796" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C796" t="inlineStr">
@@ -79989,7 +79999,7 @@
       </c>
       <c r="F796" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G796" t="n">
@@ -80010,20 +80020,24 @@
       </c>
       <c r="K796" t="inlineStr"/>
       <c r="L796" s="1" t="n">
-        <v>46202</v>
-      </c>
-      <c r="M796" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="M796" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
       <c r="N796" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O796" t="n">
-        <v>17399327</v>
+        <v>18076566</v>
       </c>
       <c r="P796" t="inlineStr">
         <is>
-          <t>Sergio Fernandes</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="Q796" t="inlineStr">
@@ -80033,16 +80047,16 @@
       </c>
       <c r="R796" t="inlineStr"/>
       <c r="S796" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="T796" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U796" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 30/06/2026 18:03:37. - Data Comentário: 30/06/2026 18:02</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/05/2026 11:16:37. - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V796" t="inlineStr"/>
@@ -80054,12 +80068,12 @@
       <c r="AB796" t="inlineStr"/>
       <c r="AC796" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 18:02</t>
+          <t>Tarefa reaberta e já passadas para o GO Sérgio que disse que as mesmas serão conclupidas até o fim da semana - Data Comentário: 22/06/2026 17:05</t>
         </is>
       </c>
       <c r="AD796" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="AE796" t="inlineStr">
@@ -80071,11 +80085,11 @@
     </row>
     <row r="797">
       <c r="A797" t="n">
-        <v>6224</v>
+        <v>6358</v>
       </c>
       <c r="B797" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>QUALITY INDUSTRIA E COMERCIO DE PRODUTOS PARA LIMPEZA LTDA</t>
         </is>
       </c>
       <c r="C797" t="inlineStr">
@@ -80095,7 +80109,7 @@
       </c>
       <c r="F797" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G797" t="n">
@@ -80116,24 +80130,20 @@
       </c>
       <c r="K797" t="inlineStr"/>
       <c r="L797" s="1" t="n">
-        <v>46171</v>
-      </c>
-      <c r="M797" t="inlineStr">
-        <is>
-          <t>26/06/2026</t>
-        </is>
-      </c>
+        <v>46202</v>
+      </c>
+      <c r="M797" t="inlineStr"/>
       <c r="N797" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O797" t="n">
-        <v>18076566</v>
+        <v>18074887</v>
       </c>
       <c r="P797" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Sergio Fernandes</t>
         </is>
       </c>
       <c r="Q797" t="inlineStr">
@@ -80143,16 +80153,16 @@
       </c>
       <c r="R797" t="inlineStr"/>
       <c r="S797" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="T797" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>MACHADO</t>
         </is>
       </c>
       <c r="U797" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/05/2026 11:16:37. - Data Comentário: 25/06/2026 16:00</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 01/07/2026 14:22:54. - Data Comentário: 01/07/2026 14:19</t>
         </is>
       </c>
       <c r="V797" t="inlineStr"/>
@@ -80164,12 +80174,12 @@
       <c r="AB797" t="inlineStr"/>
       <c r="AC797" t="inlineStr">
         <is>
-          <t>Tarefa reaberta e já passadas para o GO Sérgio que disse que as mesmas serão conclupidas até o fim da semana - Data Comentário: 22/06/2026 17:05</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 02/07/2026. - Data Comentário: 01/07/2026 14:19</t>
         </is>
       </c>
       <c r="AD797" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="AE797" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: 2026-07-01 17:12
</commit_message>
<xml_diff>
--- a/dados/base/goias.xlsx
+++ b/dados/base/goias.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF801"/>
+  <dimension ref="A1:AF803"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -946,7 +946,7 @@
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T9" t="inlineStr">
         <is>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T10" t="inlineStr">
         <is>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T12" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T14" t="inlineStr">
         <is>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T15" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T16" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T17" t="inlineStr">
         <is>
@@ -2246,7 +2246,7 @@
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -5441,7 +5441,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 03/07/2026 - Data Comentário: 30/06/2026 16:54</t>
+          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 03/07/2026 - Data Comentário: 01/07/2026 16:28</t>
         </is>
       </c>
       <c r="V49" t="inlineStr"/>
@@ -5517,7 +5517,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>03/07/2026</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>3. Folha, Aguardando Resumo p/ Processamento   Previsão para conclusão dia 02/07/2026 - Data Comentário: 26/06/2026 16:27</t>
+          <t>2. Folha Processada aguardando OK do cliente para finalização   Previsão para conclusão dia 03/07/2026 - Data Comentário: 01/07/2026 16:24</t>
         </is>
       </c>
       <c r="V50" t="inlineStr"/>
@@ -8231,7 +8231,11 @@
       <c r="L77" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="M77" t="inlineStr"/>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
       <c r="N77" t="inlineStr">
         <is>
           <t>06/2026</t>
@@ -8259,7 +8263,12 @@
           <t>LIMA MOTA</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 02/07/2026 
+Em contato com o cliente, o mesmo informou que enviará até amanhã 02/07 - Data Comentário: 01/07/2026 16:29</t>
+        </is>
+      </c>
       <c r="V77" t="inlineStr"/>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -22196,7 +22205,7 @@
       </c>
       <c r="K218" t="inlineStr"/>
       <c r="L218" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M218" t="inlineStr"/>
       <c r="N218" t="inlineStr">
@@ -22219,7 +22228,7 @@
       </c>
       <c r="R218" t="inlineStr"/>
       <c r="S218" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T218" t="inlineStr">
         <is>
@@ -22296,7 +22305,7 @@
       </c>
       <c r="K219" t="inlineStr"/>
       <c r="L219" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M219" t="inlineStr"/>
       <c r="N219" t="inlineStr">
@@ -22319,7 +22328,7 @@
       </c>
       <c r="R219" t="inlineStr"/>
       <c r="S219" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T219" t="inlineStr">
         <is>
@@ -22396,7 +22405,7 @@
       </c>
       <c r="K220" t="inlineStr"/>
       <c r="L220" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M220" t="inlineStr"/>
       <c r="N220" t="inlineStr">
@@ -22419,7 +22428,7 @@
       </c>
       <c r="R220" t="inlineStr"/>
       <c r="S220" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T220" t="inlineStr">
         <is>
@@ -22496,7 +22505,7 @@
       </c>
       <c r="K221" t="inlineStr"/>
       <c r="L221" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M221" t="inlineStr"/>
       <c r="N221" t="inlineStr">
@@ -22519,7 +22528,7 @@
       </c>
       <c r="R221" t="inlineStr"/>
       <c r="S221" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T221" t="inlineStr">
         <is>
@@ -22596,7 +22605,7 @@
       </c>
       <c r="K222" t="inlineStr"/>
       <c r="L222" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M222" t="inlineStr"/>
       <c r="N222" t="inlineStr">
@@ -22619,7 +22628,7 @@
       </c>
       <c r="R222" t="inlineStr"/>
       <c r="S222" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T222" t="inlineStr">
         <is>
@@ -22696,7 +22705,7 @@
       </c>
       <c r="K223" t="inlineStr"/>
       <c r="L223" s="1" t="n">
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="M223" t="inlineStr"/>
       <c r="N223" t="inlineStr">
@@ -22719,7 +22728,7 @@
       </c>
       <c r="R223" t="inlineStr"/>
       <c r="S223" t="n">
-        <v>-12</v>
+        <v>-14</v>
       </c>
       <c r="T223" t="inlineStr">
         <is>
@@ -78885,11 +78894,11 @@
     </row>
     <row r="786">
       <c r="A786" t="n">
-        <v>5617</v>
+        <v>6704</v>
       </c>
       <c r="B786" t="inlineStr">
         <is>
-          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
+          <t>TECNO COM INFORMATICA LTDA</t>
         </is>
       </c>
       <c r="C786" t="inlineStr">
@@ -78932,22 +78941,18 @@
       <c r="L786" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="M786" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
-        </is>
-      </c>
+      <c r="M786" t="inlineStr"/>
       <c r="N786" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O786" t="n">
-        <v>17407858</v>
+        <v>18096764</v>
       </c>
       <c r="P786" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q786" t="inlineStr">
@@ -78961,12 +78966,12 @@
       </c>
       <c r="T786" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U786" t="inlineStr">
         <is>
-          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 30/06/2026 - Data Comentário: 26/06/2026 14:11</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:27:33. - Data Comentário: 29/06/2026 09:26</t>
         </is>
       </c>
       <c r="V786" t="inlineStr"/>
@@ -78976,8 +78981,16 @@
       <c r="Z786" t="inlineStr"/>
       <c r="AA786" t="inlineStr"/>
       <c r="AB786" t="inlineStr"/>
-      <c r="AC786" t="inlineStr"/>
-      <c r="AD786" t="inlineStr"/>
+      <c r="AC786" t="inlineStr">
+        <is>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:26</t>
+        </is>
+      </c>
+      <c r="AD786" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
       <c r="AE786" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -78985,17 +78998,17 @@
       </c>
       <c r="AF786" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="787">
       <c r="A787" t="n">
-        <v>6224</v>
+        <v>6705</v>
       </c>
       <c r="B787" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>NARCIZO ALVES CORDEIRO</t>
         </is>
       </c>
       <c r="C787" t="inlineStr">
@@ -79005,7 +79018,7 @@
       </c>
       <c r="D787" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - SN</t>
         </is>
       </c>
       <c r="E787" t="inlineStr">
@@ -79015,11 +79028,11 @@
       </c>
       <c r="F787" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G787" t="n">
-        <v>7874</v>
+        <v>9762</v>
       </c>
       <c r="H787" t="n">
         <v>0</v>
@@ -79031,29 +79044,25 @@
       </c>
       <c r="J787" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>Movimento - Analise de Balanço Simples Nacional</t>
         </is>
       </c>
       <c r="K787" t="inlineStr"/>
       <c r="L787" s="1" t="n">
         <v>46198</v>
       </c>
-      <c r="M787" t="inlineStr">
-        <is>
-          <t>30/06/2026</t>
-        </is>
-      </c>
+      <c r="M787" t="inlineStr"/>
       <c r="N787" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O787" t="n">
-        <v>17206041</v>
+        <v>18096936</v>
       </c>
       <c r="P787" t="inlineStr">
         <is>
-          <t>Jackson Silva</t>
+          <t>Paulo Silva</t>
         </is>
       </c>
       <c r="Q787" t="inlineStr">
@@ -79067,12 +79076,12 @@
       </c>
       <c r="T787" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>TECNO COM</t>
         </is>
       </c>
       <c r="U787" t="inlineStr">
         <is>
-          <t>Atraso da Operação, processo em elaboração conforme data prevista  Previsão para conclusão dia 30/06/2026 - Data Comentário: 26/06/2026 14:11</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:24:47. - Data Comentário: 29/06/2026 09:23</t>
         </is>
       </c>
       <c r="V787" t="inlineStr"/>
@@ -79082,8 +79091,16 @@
       <c r="Z787" t="inlineStr"/>
       <c r="AA787" t="inlineStr"/>
       <c r="AB787" t="inlineStr"/>
-      <c r="AC787" t="inlineStr"/>
-      <c r="AD787" t="inlineStr"/>
+      <c r="AC787" t="inlineStr">
+        <is>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:23</t>
+        </is>
+      </c>
+      <c r="AD787" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
       <c r="AE787" t="inlineStr">
         <is>
           <t>Tarefa</t>
@@ -79091,17 +79108,17 @@
       </c>
       <c r="AF787" t="inlineStr">
         <is>
-          <t>Edileide Dias</t>
+          <t>Fernanda Araujo</t>
         </is>
       </c>
     </row>
     <row r="788">
       <c r="A788" t="n">
-        <v>6704</v>
+        <v>6279</v>
       </c>
       <c r="B788" t="inlineStr">
         <is>
-          <t>TECNO COM INFORMATICA LTDA</t>
+          <t>DIENNYFER DA S PEREIRA</t>
         </is>
       </c>
       <c r="C788" t="inlineStr">
@@ -79111,7 +79128,7 @@
       </c>
       <c r="D788" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E788" t="inlineStr">
@@ -79121,41 +79138,41 @@
       </c>
       <c r="F788" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G788" t="n">
-        <v>7874</v>
+        <v>5800</v>
       </c>
       <c r="H788" t="n">
-        <v>0</v>
+        <v>5776</v>
       </c>
       <c r="I788" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J788" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Real</t>
+          <t>CCT Lançamento Sd.508</t>
         </is>
       </c>
       <c r="K788" t="inlineStr"/>
       <c r="L788" s="1" t="n">
-        <v>46198</v>
+        <v>46203</v>
       </c>
       <c r="M788" t="inlineStr"/>
       <c r="N788" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>00/2026</t>
         </is>
       </c>
       <c r="O788" t="n">
-        <v>18096764</v>
+        <v>18087241</v>
       </c>
       <c r="P788" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Vitor Guedes</t>
         </is>
       </c>
       <c r="Q788" t="inlineStr">
@@ -79165,16 +79182,16 @@
       </c>
       <c r="R788" t="inlineStr"/>
       <c r="S788" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="T788" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t>EMPORIO DOS FRIOS</t>
         </is>
       </c>
       <c r="U788" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:27:33. - Data Comentário: 29/06/2026 09:26</t>
+          <t>8. Serviços Suspensos. - Data Comentário: 30/06/2026 17:29</t>
         </is>
       </c>
       <c r="V788" t="inlineStr"/>
@@ -79186,12 +79203,12 @@
       <c r="AB788" t="inlineStr"/>
       <c r="AC788" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:26</t>
+          <t>Aguardando liberação do sindicato - Data Comentário: 18/05/2026 17:19</t>
         </is>
       </c>
       <c r="AD788" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="AE788" t="inlineStr">
@@ -79201,17 +79218,17 @@
       </c>
       <c r="AF788" t="inlineStr">
         <is>
-          <t>Fernanda Araujo</t>
+          <t>David Bragança</t>
         </is>
       </c>
     </row>
     <row r="789">
       <c r="A789" t="n">
-        <v>6705</v>
+        <v>6627</v>
       </c>
       <c r="B789" t="inlineStr">
         <is>
-          <t>NARCIZO ALVES CORDEIRO</t>
+          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
         </is>
       </c>
       <c r="C789" t="inlineStr">
@@ -79221,12 +79238,12 @@
       </c>
       <c r="D789" t="inlineStr">
         <is>
-          <t>Federal - SN</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E789" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Vander Silva</t>
         </is>
       </c>
       <c r="F789" t="inlineStr">
@@ -79235,37 +79252,41 @@
         </is>
       </c>
       <c r="G789" t="n">
-        <v>9762</v>
+        <v>7026</v>
       </c>
       <c r="H789" t="n">
         <v>0</v>
       </c>
       <c r="I789" t="inlineStr">
         <is>
-          <t>CTB - CONTÁBIL VAREJO</t>
+          <t>EF - INDUSTRIA</t>
         </is>
       </c>
       <c r="J789" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Simples Nacional</t>
+          <t>Movimento - Sistema de Análise</t>
         </is>
       </c>
       <c r="K789" t="inlineStr"/>
       <c r="L789" s="1" t="n">
-        <v>46198</v>
-      </c>
-      <c r="M789" t="inlineStr"/>
+        <v>46167</v>
+      </c>
+      <c r="M789" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
       <c r="N789" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O789" t="n">
-        <v>18096936</v>
+        <v>18048469</v>
       </c>
       <c r="P789" t="inlineStr">
         <is>
-          <t>Paulo Silva</t>
+          <t>Denis Reis</t>
         </is>
       </c>
       <c r="Q789" t="inlineStr">
@@ -79275,16 +79296,17 @@
       </c>
       <c r="R789" t="inlineStr"/>
       <c r="S789" t="n">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="T789" t="inlineStr">
         <is>
-          <t>TECNO COM</t>
+          <t xml:space="preserve">GTG </t>
         </is>
       </c>
       <c r="U789" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/06/2026 09:24:47. - Data Comentário: 29/06/2026 09:23</t>
+          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 26/06/2026 
+OPERAÇÃO X GC VALIDANDO COM SYS ANALISE - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V789" t="inlineStr"/>
@@ -79296,12 +79318,12 @@
       <c r="AB789" t="inlineStr"/>
       <c r="AC789" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 30/06/2026. - Data Comentário: 29/06/2026 09:23</t>
+          <t>Operação e GC validando as informações errôneas no sistema de análise - Data Comentário: 24/06/2026 14:39</t>
         </is>
       </c>
       <c r="AD789" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="AE789" t="inlineStr">
@@ -79309,19 +79331,15 @@
           <t>Tarefa</t>
         </is>
       </c>
-      <c r="AF789" t="inlineStr">
-        <is>
-          <t>Fernanda Araujo</t>
-        </is>
-      </c>
+      <c r="AF789" t="inlineStr"/>
     </row>
     <row r="790">
       <c r="A790" t="n">
-        <v>6279</v>
+        <v>6224</v>
       </c>
       <c r="B790" t="inlineStr">
         <is>
-          <t>DIENNYFER DA S PEREIRA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C790" t="inlineStr">
@@ -79331,7 +79349,7 @@
       </c>
       <c r="D790" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E790" t="inlineStr">
@@ -79345,37 +79363,37 @@
         </is>
       </c>
       <c r="G790" t="n">
-        <v>5800</v>
+        <v>1802</v>
       </c>
       <c r="H790" t="n">
-        <v>5776</v>
+        <v>0</v>
       </c>
       <c r="I790" t="inlineStr">
         <is>
-          <t>DP - DEPTO. PESSOAL</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J790" t="inlineStr">
         <is>
-          <t>CCT Lançamento Sd.508</t>
+          <t>Est - ICMS RPA - CÓD. 046-2</t>
         </is>
       </c>
       <c r="K790" t="inlineStr"/>
       <c r="L790" s="1" t="n">
-        <v>46203</v>
+        <v>46182</v>
       </c>
       <c r="M790" t="inlineStr"/>
       <c r="N790" t="inlineStr">
         <is>
-          <t>00/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O790" t="n">
-        <v>18087241</v>
+        <v>17688680</v>
       </c>
       <c r="P790" t="inlineStr">
         <is>
-          <t>Vitor Guedes</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q790" t="inlineStr">
@@ -79385,16 +79403,16 @@
       </c>
       <c r="R790" t="inlineStr"/>
       <c r="S790" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="T790" t="inlineStr">
         <is>
-          <t>EMPORIO DOS FRIOS</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U790" t="inlineStr">
         <is>
-          <t>8. Serviços Suspensos. - Data Comentário: 30/06/2026 17:29</t>
+          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V790" t="inlineStr"/>
@@ -79406,32 +79424,32 @@
       <c r="AB790" t="inlineStr"/>
       <c r="AC790" t="inlineStr">
         <is>
-          <t>Aguardando liberação do sindicato - Data Comentário: 18/05/2026 17:19</t>
+          <t>Atraso por parte do cliente, GC e GM acionado - CA03 - Data Comentário: 25/06/2026 18:14</t>
         </is>
       </c>
       <c r="AD790" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="AE790" t="inlineStr">
         <is>
-          <t>Tarefa</t>
+          <t>Imposto</t>
         </is>
       </c>
       <c r="AF790" t="inlineStr">
         <is>
-          <t>David Bragança</t>
+          <t>Ricardo Fischer</t>
         </is>
       </c>
     </row>
     <row r="791">
       <c r="A791" t="n">
-        <v>6627</v>
+        <v>6224</v>
       </c>
       <c r="B791" t="inlineStr">
         <is>
-          <t>GTG EMPREENDIMENTOS SERVIÇOS E COMERCIO LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C791" t="inlineStr">
@@ -79446,50 +79464,46 @@
       </c>
       <c r="E791" t="inlineStr">
         <is>
-          <t>Vander Silva</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="F791" t="inlineStr">
         <is>
-          <t>Edimir Santos</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G791" t="n">
-        <v>7026</v>
+        <v>1808</v>
       </c>
       <c r="H791" t="n">
         <v>0</v>
       </c>
       <c r="I791" t="inlineStr">
         <is>
-          <t>EF - INDUSTRIA</t>
+          <t>EF - VAREJO</t>
         </is>
       </c>
       <c r="J791" t="inlineStr">
         <is>
-          <t>Movimento - Sistema de Análise</t>
+          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
         </is>
       </c>
       <c r="K791" t="inlineStr"/>
       <c r="L791" s="1" t="n">
-        <v>46167</v>
-      </c>
-      <c r="M791" t="inlineStr">
-        <is>
-          <t>26/06/2026</t>
-        </is>
-      </c>
+        <v>46195</v>
+      </c>
+      <c r="M791" t="inlineStr"/>
       <c r="N791" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O791" t="n">
-        <v>18048469</v>
+        <v>17688690</v>
       </c>
       <c r="P791" t="inlineStr">
         <is>
-          <t>Denis Reis</t>
+          <t>Cristina Leite</t>
         </is>
       </c>
       <c r="Q791" t="inlineStr">
@@ -79499,17 +79513,16 @@
       </c>
       <c r="R791" t="inlineStr"/>
       <c r="S791" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="T791" t="inlineStr">
         <is>
-          <t xml:space="preserve">GTG </t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U791" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão   Previsão para conclusão dia 26/06/2026 
-OPERAÇÃO X GC VALIDANDO COM SYS ANALISE - Data Comentário: 25/06/2026 16:00</t>
+          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
         </is>
       </c>
       <c r="V791" t="inlineStr"/>
@@ -79521,7 +79534,7 @@
       <c r="AB791" t="inlineStr"/>
       <c r="AC791" t="inlineStr">
         <is>
-          <t>Operação e GC validando as informações errôneas no sistema de análise - Data Comentário: 24/06/2026 14:39</t>
+          <t>Atraso por parte do cliente, GC e GM acionados - Data Comentário: 25/06/2026 18:14</t>
         </is>
       </c>
       <c r="AD791" t="inlineStr">
@@ -79531,18 +79544,22 @@
       </c>
       <c r="AE791" t="inlineStr">
         <is>
-          <t>Tarefa</t>
-        </is>
-      </c>
-      <c r="AF791" t="inlineStr"/>
+          <t>Imposto</t>
+        </is>
+      </c>
+      <c r="AF791" t="inlineStr">
+        <is>
+          <t>Ricardo Fischer</t>
+        </is>
+      </c>
     </row>
     <row r="792">
       <c r="A792" t="n">
-        <v>6224</v>
+        <v>6404</v>
       </c>
       <c r="B792" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>SOLAR INVESTIMENTOS LTDA</t>
         </is>
       </c>
       <c r="C792" t="inlineStr">
@@ -79552,7 +79569,7 @@
       </c>
       <c r="D792" t="inlineStr">
         <is>
-          <t>Federal - L Real -Trimestral</t>
+          <t>Federal - Lucro Presumido</t>
         </is>
       </c>
       <c r="E792" t="inlineStr">
@@ -79562,41 +79579,45 @@
       </c>
       <c r="F792" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Edimir Santos</t>
         </is>
       </c>
       <c r="G792" t="n">
-        <v>1802</v>
+        <v>11001</v>
       </c>
       <c r="H792" t="n">
         <v>0</v>
       </c>
       <c r="I792" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J792" t="inlineStr">
         <is>
-          <t>Est - ICMS RPA - CÓD. 046-2</t>
+          <t>Movimento - Analise de Balanço Lucro Presumido</t>
         </is>
       </c>
       <c r="K792" t="inlineStr"/>
       <c r="L792" s="1" t="n">
-        <v>46182</v>
-      </c>
-      <c r="M792" t="inlineStr"/>
+        <v>46202</v>
+      </c>
+      <c r="M792" t="inlineStr">
+        <is>
+          <t>02/07/2026</t>
+        </is>
+      </c>
       <c r="N792" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O792" t="n">
-        <v>17688680</v>
+        <v>16962451</v>
       </c>
       <c r="P792" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="Q792" t="inlineStr">
@@ -79606,16 +79627,17 @@
       </c>
       <c r="R792" t="inlineStr"/>
       <c r="S792" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="T792" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>SOLAR INVESTIMENTOS</t>
         </is>
       </c>
       <c r="U792" t="inlineStr">
         <is>
-          <t>Atraso do Cliente, cobrança ativa, GC e GM ciente do atraso - Data Comentário: 25/06/2026 16:00</t>
+          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
+Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
         </is>
       </c>
       <c r="V792" t="inlineStr"/>
@@ -79627,32 +79649,28 @@
       <c r="AB792" t="inlineStr"/>
       <c r="AC792" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionado - CA03 - Data Comentário: 25/06/2026 18:14</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:45</t>
         </is>
       </c>
       <c r="AD792" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="AE792" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AF792" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AF792" t="inlineStr"/>
     </row>
     <row r="793">
       <c r="A793" t="n">
-        <v>6224</v>
+        <v>5417</v>
       </c>
       <c r="B793" t="inlineStr">
         <is>
-          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C793" t="inlineStr">
@@ -79672,28 +79690,28 @@
       </c>
       <c r="F793" t="inlineStr">
         <is>
-          <t>Sem Master</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G793" t="n">
-        <v>1808</v>
+        <v>7877</v>
       </c>
       <c r="H793" t="n">
         <v>0</v>
       </c>
       <c r="I793" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>GERENCIA DE CONTAS</t>
         </is>
       </c>
       <c r="J793" t="inlineStr">
         <is>
-          <t>Fed - PIS/COFINS Não Cumul/Mon - 5856</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K793" t="inlineStr"/>
       <c r="L793" s="1" t="n">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="M793" t="inlineStr"/>
       <c r="N793" t="inlineStr">
@@ -79702,11 +79720,11 @@
         </is>
       </c>
       <c r="O793" t="n">
-        <v>17688690</v>
+        <v>17399327</v>
       </c>
       <c r="P793" t="inlineStr">
         <is>
-          <t>Cristina Leite</t>
+          <t>Sergio Fernandes</t>
         </is>
       </c>
       <c r="Q793" t="inlineStr">
@@ -79716,16 +79734,16 @@
       </c>
       <c r="R793" t="inlineStr"/>
       <c r="S793" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="T793" t="inlineStr">
         <is>
-          <t>SUPER MAIS DO GOIÁS</t>
+          <t>NOSSO NOVO SUPERMERCADO</t>
         </is>
       </c>
       <c r="U793" t="inlineStr">
         <is>
-          <t>Atraso de envio do cliente, consultar pendências no check list - Data Comentário: 23/06/2026 15:41</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 30/06/2026 18:03:37. - Data Comentário: 30/06/2026 18:02</t>
         </is>
       </c>
       <c r="V793" t="inlineStr"/>
@@ -79737,32 +79755,28 @@
       <c r="AB793" t="inlineStr"/>
       <c r="AC793" t="inlineStr">
         <is>
-          <t>Atraso por parte do cliente, GC e GM acionados - Data Comentário: 25/06/2026 18:14</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 18:02</t>
         </is>
       </c>
       <c r="AD793" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>01/07/2026</t>
         </is>
       </c>
       <c r="AE793" t="inlineStr">
         <is>
-          <t>Imposto</t>
-        </is>
-      </c>
-      <c r="AF793" t="inlineStr">
-        <is>
-          <t>Ricardo Fischer</t>
-        </is>
-      </c>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AF793" t="inlineStr"/>
     </row>
     <row r="794">
       <c r="A794" t="n">
-        <v>6404</v>
+        <v>5617</v>
       </c>
       <c r="B794" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS LTDA</t>
+          <t>SUPERMERCADO PRECO BAIXO TODO DIA LTDA</t>
         </is>
       </c>
       <c r="C794" t="inlineStr">
@@ -79772,7 +79786,7 @@
       </c>
       <c r="D794" t="inlineStr">
         <is>
-          <t>Federal - Lucro Presumido</t>
+          <t>Federal - L Real -Trimestral</t>
         </is>
       </c>
       <c r="E794" t="inlineStr">
@@ -79786,7 +79800,7 @@
         </is>
       </c>
       <c r="G794" t="n">
-        <v>11001</v>
+        <v>7877</v>
       </c>
       <c r="H794" t="n">
         <v>0</v>
@@ -79798,29 +79812,25 @@
       </c>
       <c r="J794" t="inlineStr">
         <is>
-          <t>Movimento - Analise de Balanço Lucro Presumido</t>
+          <t>Movimento - Analise de Balanço Lucro Real</t>
         </is>
       </c>
       <c r="K794" t="inlineStr"/>
       <c r="L794" s="1" t="n">
         <v>46202</v>
       </c>
-      <c r="M794" t="inlineStr">
-        <is>
-          <t>02/07/2026</t>
-        </is>
-      </c>
+      <c r="M794" t="inlineStr"/>
       <c r="N794" t="inlineStr">
         <is>
           <t>05/2026</t>
         </is>
       </c>
       <c r="O794" t="n">
-        <v>16962451</v>
+        <v>18076497</v>
       </c>
       <c r="P794" t="inlineStr">
         <is>
-          <t>Ricardo Ferreira</t>
+          <t>Sergio Fernandes</t>
         </is>
       </c>
       <c r="Q794" t="inlineStr">
@@ -79834,13 +79844,12 @@
       </c>
       <c r="T794" t="inlineStr">
         <is>
-          <t>SOLAR INVESTIMENTOS</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U794" t="inlineStr">
         <is>
-          <t>Comentário Colaborador + Previsão De Conclusão  Previsão para conclusão dia 02/07/2026 
-Analisar até 02/07/2026 - Data Comentário: 01/07/2026 07:26</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 01/07/2026 15:44:06. - Data Comentário: 01/07/2026 15:44</t>
         </is>
       </c>
       <c r="V794" t="inlineStr"/>
@@ -79852,12 +79861,12 @@
       <c r="AB794" t="inlineStr"/>
       <c r="AC794" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 08:45</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 02/07/2026. - Data Comentário: 01/07/2026 15:44</t>
         </is>
       </c>
       <c r="AD794" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="AE794" t="inlineStr">
@@ -79869,11 +79878,11 @@
     </row>
     <row r="795">
       <c r="A795" t="n">
-        <v>5417</v>
+        <v>6224</v>
       </c>
       <c r="B795" t="inlineStr">
         <is>
-          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
+          <t>VIEIRA E REZENDE TEND TUDO LTDA</t>
         </is>
       </c>
       <c r="C795" t="inlineStr">
@@ -79893,7 +79902,7 @@
       </c>
       <c r="F795" t="inlineStr">
         <is>
-          <t>Claudio Correa</t>
+          <t>Sem Master</t>
         </is>
       </c>
       <c r="G795" t="n">
@@ -79914,20 +79923,24 @@
       </c>
       <c r="K795" t="inlineStr"/>
       <c r="L795" s="1" t="n">
-        <v>46202</v>
-      </c>
-      <c r="M795" t="inlineStr"/>
+        <v>46171</v>
+      </c>
+      <c r="M795" t="inlineStr">
+        <is>
+          <t>26/06/2026</t>
+        </is>
+      </c>
       <c r="N795" t="inlineStr">
         <is>
-          <t>05/2026</t>
+          <t>04/2026</t>
         </is>
       </c>
       <c r="O795" t="n">
-        <v>17399327</v>
+        <v>18076566</v>
       </c>
       <c r="P795" t="inlineStr">
         <is>
-          <t>Sergio Fernandes</t>
+          <t>Ricardo Ferreira</t>
         </is>
       </c>
       <c r="Q795" t="inlineStr">
@@ -79937,16 +79950,16 @@
       </c>
       <c r="R795" t="inlineStr"/>
       <c r="S795" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="T795" t="inlineStr">
         <is>
-          <t>NOSSO NOVO SUPERMERCADO</t>
+          <t>SUPER MAIS DO GOIÁS</t>
         </is>
       </c>
       <c r="U795" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 30/06/2026 18:03:37. - Data Comentário: 30/06/2026 18:02</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 29/05/2026 11:16:37. - Data Comentário: 25/06/2026 16:00</t>
         </is>
       </c>
       <c r="V795" t="inlineStr"/>
@@ -79958,12 +79971,12 @@
       <c r="AB795" t="inlineStr"/>
       <c r="AC795" t="inlineStr">
         <is>
-          <t>Tarefa reaberta. A previsão de conclusão está prevista para 01/07/2026. - Data Comentário: 30/06/2026 18:02</t>
+          <t>Tarefa reaberta e já passadas para o GO Sérgio que disse que as mesmas serão conclupidas até o fim da semana - Data Comentário: 22/06/2026 17:05</t>
         </is>
       </c>
       <c r="AD795" t="inlineStr">
         <is>
-          <t>01/07/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="AE795" t="inlineStr">
@@ -80020,20 +80033,16 @@
       </c>
       <c r="K796" t="inlineStr"/>
       <c r="L796" s="1" t="n">
-        <v>46171</v>
-      </c>
-      <c r="M796" t="inlineStr">
-        <is>
-          <t>26/06/2026</t>
-        </is>
-      </c>
+        <v>46202</v>
+      </c>
+      <c r="M796" t="inlineStr"/>
       <c r="N796" t="inlineStr">
         <is>
-          <t>04/2026</t>
+          <t>05/2026</t>
         </is>
       </c>
       <c r="O796" t="n">
-        <v>18076566</v>
+        <v>18076567</v>
       </c>
       <c r="P796" t="inlineStr">
         <is>
@@ -80047,7 +80056,7 @@
       </c>
       <c r="R796" t="inlineStr"/>
       <c r="S796" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="T796" t="inlineStr">
         <is>
@@ -80056,7 +80065,7 @@
       </c>
       <c r="U796" t="inlineStr">
         <is>
-          <t>Reaberto via API integração MGC x Analise Balanço em 29/05/2026 11:16:37. - Data Comentário: 25/06/2026 16:00</t>
+          <t>Reaberto via API integração MGC x Analise Balanço em 01/07/2026 15:36:41. - Data Comentário: 01/07/2026 15:37</t>
         </is>
       </c>
       <c r="V796" t="inlineStr"/>
@@ -80068,12 +80077,12 @@
       <c r="AB796" t="inlineStr"/>
       <c r="AC796" t="inlineStr">
         <is>
-          <t>Tarefa reaberta e já passadas para o GO Sérgio que disse que as mesmas serão conclupidas até o fim da semana - Data Comentário: 22/06/2026 17:05</t>
+          <t>Tarefa reaberta. A previsão de conclusão está prevista para 02/07/2026. - Data Comentário: 01/07/2026 15:37</t>
         </is>
       </c>
       <c r="AD796" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="AE796" t="inlineStr">
@@ -80400,11 +80409,11 @@
     </row>
     <row r="800">
       <c r="A800" t="n">
-        <v>6981</v>
+        <v>5417</v>
       </c>
       <c r="B800" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C800" t="inlineStr">
@@ -80424,11 +80433,11 @@
       </c>
       <c r="F800" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G800" t="n">
-        <v>11616</v>
+        <v>11815</v>
       </c>
       <c r="H800" t="n">
         <v>0</v>
@@ -80440,7 +80449,7 @@
       </c>
       <c r="J800" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - DP - SP</t>
+          <t>Cálculo de férias individuais - ERICA MIRELE DA SILVA</t>
         </is>
       </c>
       <c r="K800" t="inlineStr"/>
@@ -80454,11 +80463,11 @@
         </is>
       </c>
       <c r="O800" t="n">
-        <v>18195071</v>
+        <v>18196300</v>
       </c>
       <c r="P800" t="inlineStr">
         <is>
-          <t>Mauricio Lermen</t>
+          <t>Mikael Teixeira</t>
         </is>
       </c>
       <c r="Q800" t="inlineStr">
@@ -80472,14 +80481,10 @@
       </c>
       <c r="T800" t="inlineStr">
         <is>
-          <t>SUPERMERCADO AVENIDA</t>
-        </is>
-      </c>
-      <c r="U800" t="inlineStr">
-        <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6981; Tarefa Incluida: 11616; Vencimento: 01/07/2026 00:00:00; UsuarioResponsavel: mauricio - Data Comentário: 01/07/2026 09:04</t>
-        </is>
-      </c>
+          <t>NOSSO NOVO SUPERMERCADO</t>
+        </is>
+      </c>
+      <c r="U800" t="inlineStr"/>
       <c r="V800" t="inlineStr"/>
       <c r="W800" t="inlineStr"/>
       <c r="X800" t="inlineStr"/>
@@ -80498,11 +80503,11 @@
     </row>
     <row r="801">
       <c r="A801" t="n">
-        <v>6981</v>
+        <v>5417</v>
       </c>
       <c r="B801" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+          <t>COMERCIAL DE ALIMENTOS ALLEGRA LTDA</t>
         </is>
       </c>
       <c r="C801" t="inlineStr">
@@ -80522,23 +80527,23 @@
       </c>
       <c r="F801" t="inlineStr">
         <is>
-          <t>Reynaldo Santos</t>
+          <t>Claudio Correa</t>
         </is>
       </c>
       <c r="G801" t="n">
-        <v>11618</v>
+        <v>11815</v>
       </c>
       <c r="H801" t="n">
         <v>0</v>
       </c>
       <c r="I801" t="inlineStr">
         <is>
-          <t>EF - VAREJO</t>
+          <t>DP - DEPTO. PESSOAL</t>
         </is>
       </c>
       <c r="J801" t="inlineStr">
         <is>
-          <t>Envio de ATA de Implantação - EF V - SP</t>
+          <t>Cálculo de férias individuais - PEDRO HENRIQUE LIMA ANDRADE</t>
         </is>
       </c>
       <c r="K801" t="inlineStr"/>
@@ -80552,11 +80557,11 @@
         </is>
       </c>
       <c r="O801" t="n">
-        <v>18195073</v>
+        <v>18196299</v>
       </c>
       <c r="P801" t="inlineStr">
         <is>
-          <t>Claudineia Rodrigues</t>
+          <t>Mikael Teixeira</t>
         </is>
       </c>
       <c r="Q801" t="inlineStr">
@@ -80570,14 +80575,10 @@
       </c>
       <c r="T801" t="inlineStr">
         <is>
-          <t>SUPERMERCADO AVENIDA</t>
-        </is>
-      </c>
-      <c r="U801" t="inlineStr">
-        <is>
-          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6981; Tarefa Incluida: 11618; Vencimento: 01/07/2026 00:00:00; UsuarioResponsavel: Claudineia - Data Comentário: 01/07/2026 09:04</t>
-        </is>
-      </c>
+          <t>NOSSO NOVO SUPERMERCADO</t>
+        </is>
+      </c>
+      <c r="U801" t="inlineStr"/>
       <c r="V801" t="inlineStr"/>
       <c r="W801" t="inlineStr"/>
       <c r="X801" t="inlineStr"/>
@@ -80594,6 +80595,202 @@
       </c>
       <c r="AF801" t="inlineStr"/>
     </row>
+    <row r="802">
+      <c r="A802" t="n">
+        <v>6981</v>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Federal - L Real -Trimestral</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G802" t="n">
+        <v>11616</v>
+      </c>
+      <c r="H802" t="n">
+        <v>0</v>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>DP - DEPTO. PESSOAL</t>
+        </is>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - DP - SP</t>
+        </is>
+      </c>
+      <c r="K802" t="inlineStr"/>
+      <c r="L802" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="M802" t="inlineStr"/>
+      <c r="N802" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O802" t="n">
+        <v>18195071</v>
+      </c>
+      <c r="P802" t="inlineStr">
+        <is>
+          <t>Mauricio Lermen</t>
+        </is>
+      </c>
+      <c r="Q802" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R802" t="inlineStr"/>
+      <c r="S802" t="n">
+        <v>0</v>
+      </c>
+      <c r="T802" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO AVENIDA</t>
+        </is>
+      </c>
+      <c r="U802" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6981; Tarefa Incluida: 11616; Vencimento: 01/07/2026 00:00:00; UsuarioResponsavel: mauricio - Data Comentário: 01/07/2026 09:04</t>
+        </is>
+      </c>
+      <c r="V802" t="inlineStr"/>
+      <c r="W802" t="inlineStr"/>
+      <c r="X802" t="inlineStr"/>
+      <c r="Y802" t="inlineStr"/>
+      <c r="Z802" t="inlineStr"/>
+      <c r="AA802" t="inlineStr"/>
+      <c r="AB802" t="inlineStr"/>
+      <c r="AC802" t="inlineStr"/>
+      <c r="AD802" t="inlineStr"/>
+      <c r="AE802" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AF802" t="inlineStr"/>
+    </row>
+    <row r="803">
+      <c r="A803" t="n">
+        <v>6981</v>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUIZ GOMES DA SILVA - O GOIANO </t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>GOIAS</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Federal - L Real -Trimestral</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>Ricardo Ferreira</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Reynaldo Santos</t>
+        </is>
+      </c>
+      <c r="G803" t="n">
+        <v>11618</v>
+      </c>
+      <c r="H803" t="n">
+        <v>0</v>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>EF - VAREJO</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>Envio de ATA de Implantação - EF V - SP</t>
+        </is>
+      </c>
+      <c r="K803" t="inlineStr"/>
+      <c r="L803" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="M803" t="inlineStr"/>
+      <c r="N803" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="O803" t="n">
+        <v>18195073</v>
+      </c>
+      <c r="P803" t="inlineStr">
+        <is>
+          <t>Claudineia Rodrigues</t>
+        </is>
+      </c>
+      <c r="Q803" t="inlineStr">
+        <is>
+          <t>Em Aberto</t>
+        </is>
+      </c>
+      <c r="R803" t="inlineStr"/>
+      <c r="S803" t="n">
+        <v>0</v>
+      </c>
+      <c r="T803" t="inlineStr">
+        <is>
+          <t>SUPERMERCADO AVENIDA</t>
+        </is>
+      </c>
+      <c r="U803" t="inlineStr">
+        <is>
+          <t>Rotina Para Criar Tarefas Dos Clientes Novos - CodCliente: 6981; Tarefa Incluida: 11618; Vencimento: 01/07/2026 00:00:00; UsuarioResponsavel: Claudineia - Data Comentário: 01/07/2026 09:04</t>
+        </is>
+      </c>
+      <c r="V803" t="inlineStr"/>
+      <c r="W803" t="inlineStr"/>
+      <c r="X803" t="inlineStr"/>
+      <c r="Y803" t="inlineStr"/>
+      <c r="Z803" t="inlineStr"/>
+      <c r="AA803" t="inlineStr"/>
+      <c r="AB803" t="inlineStr"/>
+      <c r="AC803" t="inlineStr"/>
+      <c r="AD803" t="inlineStr"/>
+      <c r="AE803" t="inlineStr">
+        <is>
+          <t>Tarefa</t>
+        </is>
+      </c>
+      <c r="AF803" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>